<commit_message>
Registra si asiste a reunion
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/formato-gdr.xlsx
+++ b/src/main/resources/templates/formato-gdr.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\ESSALUD\PROYECTOS\PROYECTO MARCACIONES\servicio-marcaciones\src\main\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7B7460B-A056-4A13-BA60-E79A17DC7F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2CF63FB-4D0F-4CFF-B8E4-41B691BB8113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -362,7 +362,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="49">
   <si>
     <t>DATOS GENERALES</t>
   </si>
@@ -1382,7 +1382,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="131">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1442,261 +1442,6 @@
     <xf numFmtId="9" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1767,6 +1512,14 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1788,7 +1541,253 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
@@ -2331,23 +2330,23 @@
       <c r="N1" s="1"/>
     </row>
     <row r="2" spans="2:14" ht="64.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="97" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="56" t="s">
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="98"/>
+      <c r="L2" s="99"/>
+      <c r="M2" s="100" t="s">
         <v>39</v>
       </c>
-      <c r="N2" s="57"/>
+      <c r="N2" s="101"/>
     </row>
     <row r="3" spans="2:14" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="3"/>
@@ -2365,21 +2364,21 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4" spans="2:14" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="102" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="59"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="60"/>
-      <c r="H4" s="60"/>
-      <c r="I4" s="60"/>
-      <c r="J4" s="60"/>
-      <c r="K4" s="60"/>
-      <c r="L4" s="60"/>
-      <c r="M4" s="60"/>
-      <c r="N4" s="61"/>
+      <c r="C4" s="103"/>
+      <c r="D4" s="104"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="104"/>
+      <c r="H4" s="104"/>
+      <c r="I4" s="104"/>
+      <c r="J4" s="104"/>
+      <c r="K4" s="104"/>
+      <c r="L4" s="104"/>
+      <c r="M4" s="104"/>
+      <c r="N4" s="105"/>
     </row>
     <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="5"/>
@@ -2397,175 +2396,175 @@
       <c r="N5" s="6"/>
     </row>
     <row r="6" spans="2:14" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="106" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="63"/>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="63"/>
-      <c r="I6" s="63"/>
-      <c r="J6" s="63"/>
-      <c r="K6" s="63"/>
-      <c r="L6" s="63"/>
-      <c r="M6" s="63"/>
-      <c r="N6" s="64"/>
+      <c r="C6" s="107"/>
+      <c r="D6" s="107"/>
+      <c r="E6" s="107"/>
+      <c r="F6" s="107"/>
+      <c r="G6" s="107"/>
+      <c r="H6" s="107"/>
+      <c r="I6" s="107"/>
+      <c r="J6" s="107"/>
+      <c r="K6" s="107"/>
+      <c r="L6" s="107"/>
+      <c r="M6" s="107"/>
+      <c r="N6" s="108"/>
     </row>
     <row r="7" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="65" t="s">
+      <c r="B7" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="66"/>
-      <c r="D7" s="66"/>
-      <c r="E7" s="66"/>
-      <c r="F7" s="66"/>
-      <c r="G7" s="67"/>
-      <c r="H7" s="65" t="s">
+      <c r="C7" s="85"/>
+      <c r="D7" s="85"/>
+      <c r="E7" s="85"/>
+      <c r="F7" s="85"/>
+      <c r="G7" s="86"/>
+      <c r="H7" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="66"/>
-      <c r="J7" s="66"/>
-      <c r="K7" s="66"/>
-      <c r="L7" s="66"/>
-      <c r="M7" s="66"/>
-      <c r="N7" s="67"/>
+      <c r="I7" s="85"/>
+      <c r="J7" s="85"/>
+      <c r="K7" s="85"/>
+      <c r="L7" s="85"/>
+      <c r="M7" s="85"/>
+      <c r="N7" s="86"/>
     </row>
     <row r="8" spans="2:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="70" t="s">
+      <c r="B8" s="61" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="71"/>
-      <c r="D8" s="74"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="75"/>
-      <c r="G8" s="76"/>
-      <c r="H8" s="26" t="s">
+      <c r="C8" s="62"/>
+      <c r="D8" s="94"/>
+      <c r="E8" s="95"/>
+      <c r="F8" s="95"/>
+      <c r="G8" s="96"/>
+      <c r="H8" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="27"/>
-      <c r="J8" s="28"/>
-      <c r="K8" s="29"/>
-      <c r="L8" s="29"/>
-      <c r="M8" s="29"/>
-      <c r="N8" s="30"/>
+      <c r="I8" s="57"/>
+      <c r="J8" s="58"/>
+      <c r="K8" s="59"/>
+      <c r="L8" s="59"/>
+      <c r="M8" s="59"/>
+      <c r="N8" s="60"/>
     </row>
     <row r="9" spans="2:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="70" t="s">
+      <c r="B9" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="71"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="26" t="s">
+      <c r="C9" s="62"/>
+      <c r="D9" s="89"/>
+      <c r="E9" s="90"/>
+      <c r="F9" s="90"/>
+      <c r="G9" s="91"/>
+      <c r="H9" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="I9" s="27"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="29"/>
-      <c r="L9" s="29"/>
-      <c r="M9" s="29"/>
-      <c r="N9" s="30"/>
+      <c r="I9" s="57"/>
+      <c r="J9" s="58"/>
+      <c r="K9" s="59"/>
+      <c r="L9" s="59"/>
+      <c r="M9" s="59"/>
+      <c r="N9" s="60"/>
     </row>
     <row r="10" spans="2:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="68" t="s">
+      <c r="B10" s="87" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="69"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="68" t="s">
+      <c r="C10" s="88"/>
+      <c r="D10" s="89"/>
+      <c r="E10" s="90"/>
+      <c r="F10" s="90"/>
+      <c r="G10" s="91"/>
+      <c r="H10" s="87" t="s">
         <v>9</v>
       </c>
-      <c r="I10" s="69"/>
-      <c r="J10" s="69"/>
-      <c r="K10" s="29"/>
-      <c r="L10" s="29"/>
-      <c r="M10" s="29"/>
-      <c r="N10" s="30"/>
+      <c r="I10" s="88"/>
+      <c r="J10" s="88"/>
+      <c r="K10" s="59"/>
+      <c r="L10" s="59"/>
+      <c r="M10" s="59"/>
+      <c r="N10" s="60"/>
     </row>
     <row r="11" spans="2:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="70" t="s">
+      <c r="B11" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="71"/>
-      <c r="D11" s="23" t="s">
+      <c r="C11" s="62"/>
+      <c r="D11" s="89" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="68" t="s">
+      <c r="E11" s="90"/>
+      <c r="F11" s="90"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="87" t="s">
         <v>10</v>
       </c>
-      <c r="I11" s="69"/>
-      <c r="J11" s="69"/>
-      <c r="K11" s="72" t="s">
+      <c r="I11" s="88"/>
+      <c r="J11" s="88"/>
+      <c r="K11" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="L11" s="72"/>
-      <c r="M11" s="72"/>
-      <c r="N11" s="73"/>
+      <c r="L11" s="92"/>
+      <c r="M11" s="92"/>
+      <c r="N11" s="93"/>
     </row>
     <row r="12" spans="2:14" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="68" t="s">
+      <c r="B12" s="87" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="69"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="68" t="s">
+      <c r="C12" s="88"/>
+      <c r="D12" s="89"/>
+      <c r="E12" s="90"/>
+      <c r="F12" s="90"/>
+      <c r="G12" s="91"/>
+      <c r="H12" s="87" t="s">
         <v>11</v>
       </c>
-      <c r="I12" s="69"/>
-      <c r="J12" s="69"/>
-      <c r="K12" s="29"/>
-      <c r="L12" s="29"/>
-      <c r="M12" s="29"/>
-      <c r="N12" s="30"/>
+      <c r="I12" s="88"/>
+      <c r="J12" s="88"/>
+      <c r="K12" s="59"/>
+      <c r="L12" s="59"/>
+      <c r="M12" s="59"/>
+      <c r="N12" s="60"/>
     </row>
     <row r="13" spans="2:14" s="20" customFormat="1" ht="71.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="19"/>
-      <c r="C13" s="38" t="s">
+      <c r="C13" s="130" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="38"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="38"/>
-      <c r="H13" s="38"/>
-      <c r="I13" s="38"/>
-      <c r="J13" s="38"/>
-      <c r="K13" s="38"/>
-      <c r="L13" s="38"/>
-      <c r="M13" s="38"/>
-      <c r="N13" s="38"/>
+      <c r="D13" s="130"/>
+      <c r="E13" s="130"/>
+      <c r="F13" s="130"/>
+      <c r="G13" s="130"/>
+      <c r="H13" s="130"/>
+      <c r="I13" s="130"/>
+      <c r="J13" s="130"/>
+      <c r="K13" s="130"/>
+      <c r="L13" s="130"/>
+      <c r="M13" s="130"/>
+      <c r="N13" s="130"/>
     </row>
     <row r="14" spans="2:14" ht="96" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="123" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="32"/>
-      <c r="D14" s="33"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="31" t="s">
+      <c r="C14" s="124"/>
+      <c r="D14" s="125"/>
+      <c r="E14" s="126"/>
+      <c r="F14" s="126"/>
+      <c r="G14" s="127"/>
+      <c r="H14" s="123" t="s">
         <v>12</v>
       </c>
-      <c r="I14" s="32"/>
-      <c r="J14" s="32"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="37"/>
+      <c r="I14" s="124"/>
+      <c r="J14" s="124"/>
+      <c r="K14" s="128"/>
+      <c r="L14" s="128"/>
+      <c r="M14" s="128"/>
+      <c r="N14" s="129"/>
     </row>
     <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="8"/>
@@ -2583,98 +2582,96 @@
       <c r="N15" s="8"/>
     </row>
     <row r="16" spans="2:14" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="87" t="s">
+      <c r="B16" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="C16" s="88"/>
-      <c r="D16" s="88"/>
-      <c r="E16" s="88"/>
-      <c r="F16" s="88"/>
-      <c r="G16" s="88"/>
-      <c r="H16" s="88"/>
-      <c r="I16" s="88"/>
-      <c r="J16" s="88"/>
-      <c r="K16" s="88"/>
-      <c r="L16" s="88"/>
-      <c r="M16" s="88"/>
-      <c r="N16" s="89"/>
+      <c r="C16" s="69"/>
+      <c r="D16" s="69"/>
+      <c r="E16" s="69"/>
+      <c r="F16" s="69"/>
+      <c r="G16" s="69"/>
+      <c r="H16" s="69"/>
+      <c r="I16" s="69"/>
+      <c r="J16" s="69"/>
+      <c r="K16" s="69"/>
+      <c r="L16" s="69"/>
+      <c r="M16" s="69"/>
+      <c r="N16" s="70"/>
     </row>
     <row r="17" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B17" s="90" t="s">
+      <c r="B17" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="91"/>
-      <c r="D17" s="91"/>
-      <c r="E17" s="91"/>
-      <c r="F17" s="91"/>
-      <c r="G17" s="91"/>
-      <c r="H17" s="91"/>
-      <c r="I17" s="92"/>
-      <c r="J17" s="93" t="s">
+      <c r="C17" s="72"/>
+      <c r="D17" s="72"/>
+      <c r="E17" s="72"/>
+      <c r="F17" s="72"/>
+      <c r="G17" s="72"/>
+      <c r="H17" s="72"/>
+      <c r="I17" s="73"/>
+      <c r="J17" s="74" t="s">
         <v>14</v>
       </c>
-      <c r="K17" s="94"/>
-      <c r="L17" s="95"/>
-      <c r="M17" s="96" t="s">
+      <c r="K17" s="75"/>
+      <c r="L17" s="76"/>
+      <c r="M17" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="N17" s="97"/>
+      <c r="N17" s="78"/>
     </row>
     <row r="18" spans="2:14" ht="58.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="98" t="s">
+      <c r="B18" s="79" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="99"/>
-      <c r="D18" s="100" t="s">
+      <c r="C18" s="80"/>
+      <c r="D18" s="81" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="100"/>
-      <c r="F18" s="99" t="s">
+      <c r="E18" s="81"/>
+      <c r="F18" s="80" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="99"/>
-      <c r="H18" s="101" t="s">
-        <v>42</v>
-      </c>
-      <c r="I18" s="102"/>
-      <c r="J18" s="103" t="s">
+      <c r="G18" s="80"/>
+      <c r="H18" s="43"/>
+      <c r="I18" s="44"/>
+      <c r="J18" s="82" t="s">
         <v>36</v>
       </c>
-      <c r="K18" s="104"/>
+      <c r="K18" s="83"/>
       <c r="L18" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M18" s="39" t="s">
+      <c r="M18" s="109" t="s">
         <v>41</v>
       </c>
-      <c r="N18" s="42" t="s">
+      <c r="N18" s="112" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="19" spans="2:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="45" t="s">
+      <c r="B19" s="115" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="46"/>
-      <c r="D19" s="48" t="s">
+      <c r="C19" s="116"/>
+      <c r="D19" s="118" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="48"/>
-      <c r="F19" s="48"/>
-      <c r="G19" s="48"/>
-      <c r="H19" s="48"/>
-      <c r="I19" s="49"/>
-      <c r="J19" s="50" t="s">
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
+      <c r="G19" s="118"/>
+      <c r="H19" s="118"/>
+      <c r="I19" s="119"/>
+      <c r="J19" s="120" t="s">
         <v>21</v>
       </c>
-      <c r="K19" s="51"/>
-      <c r="L19" s="52"/>
-      <c r="M19" s="40"/>
-      <c r="N19" s="43"/>
+      <c r="K19" s="121"/>
+      <c r="L19" s="122"/>
+      <c r="M19" s="110"/>
+      <c r="N19" s="113"/>
     </row>
     <row r="20" spans="2:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="B20" s="47"/>
-      <c r="C20" s="46"/>
+      <c r="B20" s="117"/>
+      <c r="C20" s="116"/>
       <c r="D20" s="11" t="s">
         <v>22</v>
       </c>
@@ -2693,13 +2690,13 @@
       <c r="I20" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="J20" s="50" t="s">
+      <c r="J20" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="K20" s="51"/>
-      <c r="L20" s="52"/>
-      <c r="M20" s="41"/>
-      <c r="N20" s="44"/>
+      <c r="K20" s="121"/>
+      <c r="L20" s="122"/>
+      <c r="M20" s="111"/>
+      <c r="N20" s="114"/>
     </row>
     <row r="21" spans="2:14" ht="23.25" x14ac:dyDescent="0.25">
       <c r="B21" s="13"/>
@@ -2732,147 +2729,147 @@
       <c r="N22" s="6"/>
     </row>
     <row r="23" spans="2:14" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="82" t="s">
+      <c r="B23" s="63" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="83"/>
-      <c r="D23" s="84" t="s">
+      <c r="C23" s="64"/>
+      <c r="D23" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="E23" s="85"/>
-      <c r="F23" s="85"/>
-      <c r="G23" s="85"/>
-      <c r="H23" s="85"/>
-      <c r="I23" s="85"/>
-      <c r="J23" s="85"/>
-      <c r="K23" s="85"/>
-      <c r="L23" s="85"/>
-      <c r="M23" s="85"/>
-      <c r="N23" s="86"/>
+      <c r="E23" s="66"/>
+      <c r="F23" s="66"/>
+      <c r="G23" s="66"/>
+      <c r="H23" s="66"/>
+      <c r="I23" s="66"/>
+      <c r="J23" s="66"/>
+      <c r="K23" s="66"/>
+      <c r="L23" s="66"/>
+      <c r="M23" s="66"/>
+      <c r="N23" s="67"/>
     </row>
     <row r="24" spans="2:14" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="110" t="s">
+      <c r="B24" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="111"/>
-      <c r="D24" s="112" t="s">
+      <c r="C24" s="29"/>
+      <c r="D24" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="E24" s="113"/>
-      <c r="F24" s="113"/>
-      <c r="G24" s="113" t="s">
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="H24" s="113"/>
-      <c r="I24" s="113" t="s">
+      <c r="H24" s="31"/>
+      <c r="I24" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="J24" s="113"/>
-      <c r="K24" s="113"/>
-      <c r="L24" s="113"/>
-      <c r="M24" s="114" t="s">
+      <c r="J24" s="31"/>
+      <c r="K24" s="31"/>
+      <c r="L24" s="31"/>
+      <c r="M24" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="N24" s="115"/>
+      <c r="N24" s="33"/>
     </row>
     <row r="25" spans="2:14" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="116" t="s">
+      <c r="B25" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="117"/>
-      <c r="D25" s="118"/>
-      <c r="E25" s="119"/>
-      <c r="F25" s="119"/>
-      <c r="G25" s="122" t="str">
+      <c r="C25" s="35"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
+      <c r="G25" s="40" t="str">
         <f>IF(OR(D18="No",L18="No"),"Desaprobado",IF(B25="[Seleccione]","-",IF(B25="Tiene menos de 6 meses desempeñando el puesto que es objeto de evaluación.","No corresponde calificación",IF(OR(D25="-",D11="[Seleccione]",D11="")=TRUE,"-",IF(AND(B27="Sí",D25&gt;=100),"Rendimiento Distinguido",IF(AND(D11="DIRECTIVO",D25&gt;=70),"Buen rendimiento",IF(AND(D25&gt;=60,OR(D11="MANDO MEDIO",D11="EJECUTOR",D11="OPERADOR Y DE ASISTENCIA"))=TRUE,"Buen rendimiento","Rendimiento sujeto a observación")))))))</f>
         <v>-</v>
       </c>
-      <c r="H25" s="122"/>
+      <c r="H25" s="40"/>
       <c r="I25" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="J25" s="124"/>
-      <c r="K25" s="124"/>
-      <c r="L25" s="124"/>
-      <c r="M25" s="101" t="s">
+      <c r="J25" s="42"/>
+      <c r="K25" s="42"/>
+      <c r="L25" s="42"/>
+      <c r="M25" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="N25" s="102"/>
+      <c r="N25" s="44"/>
     </row>
     <row r="26" spans="2:14" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="110" t="s">
+      <c r="B26" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="127"/>
-      <c r="D26" s="118"/>
-      <c r="E26" s="119"/>
-      <c r="F26" s="119"/>
-      <c r="G26" s="122"/>
-      <c r="H26" s="122"/>
-      <c r="I26" s="128" t="s">
+      <c r="C26" s="47"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="37"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="40"/>
+      <c r="I26" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="J26" s="124"/>
-      <c r="K26" s="124"/>
-      <c r="L26" s="124"/>
-      <c r="M26" s="101"/>
-      <c r="N26" s="102"/>
+      <c r="J26" s="42"/>
+      <c r="K26" s="42"/>
+      <c r="L26" s="42"/>
+      <c r="M26" s="43"/>
+      <c r="N26" s="44"/>
     </row>
     <row r="27" spans="2:14" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="77" t="s">
+      <c r="B27" s="51" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="78"/>
-      <c r="D27" s="120"/>
-      <c r="E27" s="121"/>
-      <c r="F27" s="121"/>
-      <c r="G27" s="123"/>
-      <c r="H27" s="123"/>
-      <c r="I27" s="129"/>
-      <c r="J27" s="130"/>
-      <c r="K27" s="130"/>
-      <c r="L27" s="130"/>
-      <c r="M27" s="125"/>
-      <c r="N27" s="126"/>
+      <c r="C27" s="52"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="41"/>
+      <c r="H27" s="41"/>
+      <c r="I27" s="49"/>
+      <c r="J27" s="50"/>
+      <c r="K27" s="50"/>
+      <c r="L27" s="50"/>
+      <c r="M27" s="45"/>
+      <c r="N27" s="46"/>
     </row>
     <row r="28" spans="2:14" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="79" t="s">
+      <c r="B28" s="53" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="80"/>
-      <c r="F28" s="80"/>
-      <c r="G28" s="80"/>
-      <c r="H28" s="80"/>
-      <c r="I28" s="80"/>
-      <c r="J28" s="80"/>
-      <c r="K28" s="80"/>
-      <c r="L28" s="80"/>
-      <c r="M28" s="80"/>
-      <c r="N28" s="81"/>
+      <c r="C28" s="54"/>
+      <c r="D28" s="54"/>
+      <c r="E28" s="54"/>
+      <c r="F28" s="54"/>
+      <c r="G28" s="54"/>
+      <c r="H28" s="54"/>
+      <c r="I28" s="54"/>
+      <c r="J28" s="54"/>
+      <c r="K28" s="54"/>
+      <c r="L28" s="54"/>
+      <c r="M28" s="54"/>
+      <c r="N28" s="55"/>
     </row>
     <row r="29" spans="2:14" ht="104.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="105" t="s">
+      <c r="B29" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="C29" s="106"/>
-      <c r="D29" s="107"/>
-      <c r="E29" s="107"/>
-      <c r="F29" s="107"/>
-      <c r="G29" s="107"/>
-      <c r="H29" s="107"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="25"/>
       <c r="I29" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="J29" s="108"/>
-      <c r="K29" s="108"/>
-      <c r="L29" s="108"/>
-      <c r="M29" s="108"/>
-      <c r="N29" s="109"/>
+      <c r="J29" s="26"/>
+      <c r="K29" s="26"/>
+      <c r="L29" s="26"/>
+      <c r="M29" s="26"/>
+      <c r="N29" s="27"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B31" s="131" t="s">
+      <c r="B31" t="s">
         <v>48</v>
       </c>
       <c r="C31" s="21"/>
@@ -2883,6 +2880,57 @@
     </row>
   </sheetData>
   <mergeCells count="67">
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="K14:N14"/>
+    <mergeCell ref="C13:N13"/>
+    <mergeCell ref="M18:M20"/>
+    <mergeCell ref="N18:N20"/>
+    <mergeCell ref="B19:C20"/>
+    <mergeCell ref="D19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:N4"/>
+    <mergeCell ref="B6:N6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="H7:N7"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="K12:N12"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="K10:N10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="K11:N11"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:N28"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:N23"/>
+    <mergeCell ref="B16:N16"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="J18:K18"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="D29:H29"/>
     <mergeCell ref="J29:N29"/>
@@ -2899,57 +2947,6 @@
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="I26:I27"/>
     <mergeCell ref="J26:L27"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:N28"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:N23"/>
-    <mergeCell ref="B16:N16"/>
-    <mergeCell ref="B17:I17"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="H7:N7"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="K12:N12"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="K11:N11"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="B2:L2"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:N4"/>
-    <mergeCell ref="B6:N6"/>
-    <mergeCell ref="M18:M20"/>
-    <mergeCell ref="N18:N20"/>
-    <mergeCell ref="B19:C20"/>
-    <mergeCell ref="D19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:L20"/>
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="K9:N9"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D14:G14"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="K14:N14"/>
-    <mergeCell ref="C13:N13"/>
   </mergeCells>
   <conditionalFormatting sqref="B25:C25">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">

</xml_diff>